<commit_message>
before removing legacy docs
</commit_message>
<xml_diff>
--- a/hypothesis_definitions.xlsx
+++ b/hypothesis_definitions.xlsx
@@ -1287,12 +1287,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1303,12 +1305,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Field Type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Required?</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Default Value</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Source/Notes</t>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>How Value is Determined</t>
         </is>
       </c>
     </row>
@@ -1320,12 +1332,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Hypothesis Only</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>not_set</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>No default - only used when hypothesis active</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Only used when testing this hypothesis</t>
         </is>
       </c>
     </row>
@@ -1337,12 +1359,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Required + Hypothesis</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>desired_outcome</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Fallback default, but varies by feature (see feature_angle mapping)</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>varies by feature (see feature mapping below)</t>
         </is>
       </c>
     </row>
@@ -1354,12 +1386,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Required + Hypothesis</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>problem_aware</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Hardcoded in persona defaults (line 1596)</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>hardcoded default</t>
         </is>
       </c>
     </row>
@@ -1371,12 +1413,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Hypothesis Only</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>not_set</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>No default - only used when hypothesis active</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Only used when testing this hypothesis</t>
         </is>
       </c>
     </row>
@@ -1388,12 +1440,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Hypothesis Only</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>not_set</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>No default - only used when hypothesis active</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Only used when testing this hypothesis</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1467,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Required + Hypothesis</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>four_us</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Fallback default, but varies by format (HERO=four_us, UGC=pas, etc.)</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>varies by format (see format mapping below)</t>
         </is>
       </c>
     </row>
@@ -1418,258 +1490,400 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Feature-based Concept Angle Defaults:</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>(used when generating without hypothesis)</t>
-        </is>
+      <c r="A9">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="B9">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>=======================================</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>am_routine</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>curiosity</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Lead with question or mechanism gap</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>pm_routine</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Lead with real-life routine narrative</t>
-        </is>
-      </c>
+          <t>FEATURE-BASED CONCEPT ANGLE (H2) - applies when NO hypothesis selected</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cravings_down</t>
+          <t>When you advertise this feature...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>pain_point</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Lead with specific problem/friction</t>
-        </is>
-      </c>
+          <t>...use this concept_angle (messaging angle)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>guided_support</t>
+          <t>am_routine (morning routine)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>social_proof</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Lead with trust, usage, testimonials</t>
-        </is>
-      </c>
+          <t>curiosity → Lead with question or mechanism gap</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>structured_system</t>
+          <t>pm_routine (evening routine)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>desired_outcome</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Lead with result or felt outcome</t>
-        </is>
-      </c>
+          <t>story → Lead with real-life routine narrative</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>homemade_food</t>
+          <t>cravings_down (hunger/cravings control)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Contrast with stricter/harder alternatives</t>
-        </is>
-      </c>
+          <t>pain_point → Lead with specific problem/friction</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>natural_safe</t>
+          <t>guided_support (support/community)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>authority</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Lead with expertise, doctor/Ayurveda credibility</t>
-        </is>
-      </c>
+          <t>social_proof → Lead with trust and testimonials</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>proof_guarantee</t>
+          <t>structured_system (the system)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>offer</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Lead with practical reason to act</t>
-        </is>
-      </c>
+          <t>desired_outcome → Lead with result or felt outcome</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>homemade_food (food aspect)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>comparison → Contrast with stricter/harder alternatives</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Format-based Concept Structure Defaults:</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>(used when generating without hypothesis)</t>
-        </is>
-      </c>
+          <t>natural_safe (natural/ayurveda)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>authority → Lead with doctor/Ayurveda credibility</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HERO</t>
+          <t>proof_guarantee (results/guarantee)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>four_us</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Default: four_us, rotation: fab, pas, bab</t>
-        </is>
-      </c>
+          <t>offer → Lead with practical reason to act</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>bab</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Default: bab, rotation: pas, fab, four_us</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>bab</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Default: bab, rotation: pas, four_us, fab</t>
-        </is>
+      <c r="A22">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="B22">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="D22">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="E22">
+        <f>=======================================</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>FEAT</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>fab</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Default: fab, rotation: four_us, pas, bab</t>
-        </is>
-      </c>
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>UGC</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>pas</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Default: pas, rotation: bab, fab, four_us</t>
-        </is>
-      </c>
+          <t>FORMAT-BASED CONCEPT STRUCTURE (H6) - applies when NO hypothesis selected</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>When you generate this format...</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>...use this concept_structure (copy flow)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>HERO (hero image)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>four_us → Useful, urgent, unique, ultra-specific</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BA (before/after)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>bab → Before → After → Bridge</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TEST (testimonial)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>bab → Before → After → Bridge</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>FEAT (features)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>fab → Feature → Advantage → Benefit</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>UGC (creator style)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>pas → Problem → Agitation → Solution</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="B32">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="C32">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="D32">
+        <f>=======================================</f>
+        <v/>
+      </c>
+      <c r="E32">
+        <f>=======================================</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>IMPORTANT: Hypothesis only affects the ONE dimension you select</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Example: Selecting concept_angle=offer ONLY changes concept_angle</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>- awareness_stage stays at default: problem_aware</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>- concept_structure stays at format rotation logic</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>